<commit_message>
Actualizacion precios e inventario
</commit_message>
<xml_diff>
--- a/inventario_agonia.xlsx
+++ b/inventario_agonia.xlsx
@@ -2,15 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -46,10 +42,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -62,9 +67,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -211,6 +216,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -245,6 +251,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -279,20 +286,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -414,7 +417,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -426,7 +468,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G161"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -836,10 +881,10 @@
         <v>7</v>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1097,10 +1142,10 @@
         <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1155,10 +1200,10 @@
         <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1358,10 +1403,10 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -3156,10 +3201,10 @@
         <v>1</v>
       </c>
       <c r="F94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3185,10 +3230,10 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -3388,10 +3433,10 @@
         <v>1</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -3816,7 +3861,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>XS</t>
+          <t>XC</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4287,10 +4332,10 @@
         <v>2</v>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G133" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -5106,6 +5151,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>